<commit_message>
lista de requisitos com a pesquisa
Nessa etapa a lista está preenchida com os requisitos funcionais e não funcionais com a pesquisa sobre ideias de MARKETPLACE DIGITAL
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/Lista de Requisitos.xlsx
+++ b/PastaDocsEngenhariaSw/Lista de Requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94c088a9ff7e7b96/Documentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFD37711-4EC0-458E-8D83-D554024EF541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{CFD37711-4EC0-458E-8D83-D554024EF541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4F645DA-4008-4822-8AE4-5F35C92F0647}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F0F0F44B-035A-4717-9A46-FD9932A1F9E0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t xml:space="preserve">LISTA DE REQUISITOS DE  MARKETPLACE DIGITAL </t>
   </si>
@@ -75,12 +75,111 @@
   <si>
     <t>Descrição da regra de domínio</t>
   </si>
+  <si>
+    <t>Rf-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ferramentas de marketing e promoção</t>
+  </si>
+  <si>
+    <t>anúncios patrocinados e campanhas promocionais.</t>
+  </si>
+  <si>
+    <t>Rf-02</t>
+  </si>
+  <si>
+    <t>Rf-03</t>
+  </si>
+  <si>
+    <t>Rf-04</t>
+  </si>
+  <si>
+    <t>Rf-05</t>
+  </si>
+  <si>
+    <t>permitir que pessoas físicas e jurídicas se cadastrem para vender.</t>
+  </si>
+  <si>
+    <t>Cadastro simplificado (CPF/CNPJ)</t>
+  </si>
+  <si>
+    <t>Integrações nativas</t>
+  </si>
+  <si>
+    <t>conexão com plataformas de e-commerce, ERPs e hubs integradores.</t>
+  </si>
+  <si>
+    <t>Sistema de reputação</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir que compradores avaliem vendedores e produtos, gerando uma pontuação de confiança.</t>
+  </si>
+  <si>
+    <t>Rf-06</t>
+  </si>
+  <si>
+    <t>Segurança de dados</t>
+  </si>
+  <si>
+    <t>O sistema deve armazenar dados pessoais e financeiros em banco de dados criptografado, garantindo conformidade com a LGPD.</t>
+  </si>
+  <si>
+    <t>Usabilidade</t>
+  </si>
+  <si>
+    <t>A interface deve ser responsiva e intuitiva, permitindo acesso via desktop e dispositivos móveis.</t>
+  </si>
+  <si>
+    <t>Gestão centralizada do operador</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir ao operador acompanhar todo o ciclo de gestão, operação, logística e financeira, incluindo indicadores de satisfação de clientes.</t>
+  </si>
+  <si>
+    <t>Rnf-01</t>
+  </si>
+  <si>
+    <t>Rnf-02</t>
+  </si>
+  <si>
+    <t>Rnf-03</t>
+  </si>
+  <si>
+    <t>Rnf-04</t>
+  </si>
+  <si>
+    <t>Rnf-05</t>
+  </si>
+  <si>
+    <t>Acessibilidade</t>
+  </si>
+  <si>
+    <t>O sistema deve seguir padrões de acessibilidade (WCAG), garantindo uso por pessoas com deficiência visual ou motora.</t>
+  </si>
+  <si>
+    <t>Escalabilidade horizontal</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir expansão de servidores e serviços em nuvem para suportar picos de acesso.</t>
+  </si>
+  <si>
+    <t>Ferramentas de Monitoramento contínuo</t>
+  </si>
+  <si>
+    <t>O sistema deve ter ferramentas de monitoramento para identificar falhas, quedas de desempenho e ataques em tempo real.</t>
+  </si>
+  <si>
+    <t>Compatibilidade multiplataforma</t>
+  </si>
+  <si>
+    <t>O sistema deve funcionar em navegadores modernos e oferecer aplicativos nativos para Android e iOS.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,6 +206,12 @@
       <b/>
       <sz val="11"/>
       <color theme="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -166,9 +271,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -503,15 +608,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C69279B-F702-4D47-A34B-1327FBBDF6C0}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="40.33203125" customWidth="1"/>
-    <col min="3" max="3" width="121.44140625" customWidth="1"/>
+    <col min="3" max="3" width="130.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -520,17 +625,14 @@
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -541,62 +643,128 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -648,7 +816,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
+      <c r="B26" s="2"/>
       <c r="C26" s="1"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -658,7 +826,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="2"/>
+      <c r="B28" s="1"/>
       <c r="C28" s="1"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -666,12 +834,8 @@
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-    </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lista de requisitos com pesquisa e brainstorm
Lista de requisitos com pesquisa e brainstorm com todos os requisitos preenchidos
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/Lista de Requisitos.xlsx
+++ b/PastaDocsEngenhariaSw/Lista de Requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94c088a9ff7e7b96/Documentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{CFD37711-4EC0-458E-8D83-D554024EF541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4F645DA-4008-4822-8AE4-5F35C92F0647}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="8_{CFD37711-4EC0-458E-8D83-D554024EF541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E58A5988-9932-4D1A-A81D-FAAE37558FB9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F0F0F44B-035A-4717-9A46-FD9932A1F9E0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t xml:space="preserve">LISTA DE REQUISITOS DE  MARKETPLACE DIGITAL </t>
   </si>
@@ -136,9 +136,6 @@
     <t>O sistema deve permitir ao operador acompanhar todo o ciclo de gestão, operação, logística e financeira, incluindo indicadores de satisfação de clientes.</t>
   </si>
   <si>
-    <t>Rnf-01</t>
-  </si>
-  <si>
     <t>Rnf-02</t>
   </si>
   <si>
@@ -173,6 +170,108 @@
   </si>
   <si>
     <t>O sistema deve funcionar em navegadores modernos e oferecer aplicativos nativos para Android e iOS.</t>
+  </si>
+  <si>
+    <t>Rf-07</t>
+  </si>
+  <si>
+    <t>Rf-08</t>
+  </si>
+  <si>
+    <t>Rf-09</t>
+  </si>
+  <si>
+    <t>Rf-10</t>
+  </si>
+  <si>
+    <t>Programa de fidelidade</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir que clientes e vendedores acumulem pontos a cada compra e venda,  e troquem por descontos ou benefícios.</t>
+  </si>
+  <si>
+    <t>Chat em tempo real</t>
+  </si>
+  <si>
+    <t>Comparação de produtos</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir que clientes comparem preços, características e avaliações de produtos lado a lado.</t>
+  </si>
+  <si>
+    <t>O sistema deve oferecer comunicação direta entre comprador e vendedor para tirar dúvidas antes da compra.</t>
+  </si>
+  <si>
+    <t>Rnf-06</t>
+  </si>
+  <si>
+    <t>Rnf-07</t>
+  </si>
+  <si>
+    <t>Rnf-08</t>
+  </si>
+  <si>
+    <t>Suporte multilíngue</t>
+  </si>
+  <si>
+    <t>O sistema deve oferecer interface em português, inglês e espanhol para ampliar alcance internacional.</t>
+  </si>
+  <si>
+    <t>Alta disponibilidade em picos de acesso</t>
+  </si>
+  <si>
+    <t>O sistema deve suportar grandes volumes de acessos simultâneos em datas especiais (Black Friday, Natal).</t>
+  </si>
+  <si>
+    <t>Convivência com sistemas legados</t>
+  </si>
+  <si>
+    <t>O sistema deve ser capaz de se integrar com softwares já existentes na empresa sem comprometer desempenho.</t>
+  </si>
+  <si>
+    <t>Rf-11</t>
+  </si>
+  <si>
+    <t>Rf-12</t>
+  </si>
+  <si>
+    <t>Gestão de devoluções e trocas</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir que clientes solicitem devoluções ou trocas, com acompanhamento do status.</t>
+  </si>
+  <si>
+    <t>Emissão de notas fiscais eletrônicas</t>
+  </si>
+  <si>
+    <t>O sistema deve gerar automaticamente NF-e conforme legislação brasileira, integrando com sistemas fiscais.</t>
+  </si>
+  <si>
+    <t>Rnf-09</t>
+  </si>
+  <si>
+    <t>Rnf-10</t>
+  </si>
+  <si>
+    <t>Rnf-11</t>
+  </si>
+  <si>
+    <t>Autenticação multifator (MFA)</t>
+  </si>
+  <si>
+    <t>O sistema deve exigir autenticação em dois passos para vendedores e administradores, aumentando a segurança.</t>
+  </si>
+  <si>
+    <t>Suporte a múltiplas moedas</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir transações em diferentes moedas, com conversão automática.</t>
+  </si>
+  <si>
+    <t>suporte técnico</t>
+  </si>
+  <si>
+    <t>O sistema deve oferecer suporte técnico com tempo máximo de resposta de 24h para incidentes críticos.</t>
   </si>
 </sst>
 </file>
@@ -217,7 +316,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -233,6 +332,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -264,16 +369,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -289,6 +397,109 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>285751</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>97155</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2693670" cy="3333220"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="CaixaDeTexto 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D82C44B4-8E8E-72C6-0F8C-AFDE100EE070}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12774931" y="828675"/>
+          <a:ext cx="2693670" cy="3333220"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent5">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400"/>
+            <a:t>- O que está grifado</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+            <a:t> de azul é o brainstorm.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" baseline="0"/>
+            <a:t>- O sites de pesquisa foram:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" baseline="0"/>
+            <a:t>1. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t>https://fcamara.com/solucoes-marketplace/ </a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100"/>
+            <a:t>2. </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t>https://venda.amazon.com.br/amazon-mentor?ld=SEBRSOA_mentor-all_go_cmp-20388875416_adg-157141521568_ad-666337958327_kwd-2278836027537_dev-c_ext-_sig-CjwKCAjw7vzOBhBxEiwAc7WNr-1Ruz3k2YRxgNfIzzAX5Nt2v5sTBED8m5OG0PTsK0nsIRQR75y23hoC8Y4QAvD_BwE&amp;gad_source=1&amp;gad_campaignid=20388875416&amp;gbraid=0AAAAAC92FE9k9c5eOd2eMSq0nOuzmyBT7&amp;gclid=CjwKCAjw7vzOBhBxEiwAc7WNr-1Ruz3k2YRxgNfIzzAX5Nt2v5sTBED8m5OG0PTsK0nsIRQR75y23hoC8Y4QAvD_BwE</a:t>
+          </a:r>
+          <a:endParaRPr lang="pt-BR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -608,38 +819,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C69279B-F702-4D47-A34B-1327FBBDF6C0}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="40.33203125" customWidth="1"/>
-    <col min="3" max="3" width="130.77734375" customWidth="1"/>
+    <col min="3" max="3" width="132.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -658,7 +869,7 @@
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -702,7 +913,7 @@
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -711,131 +922,189 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="C18" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="C19" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="B20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="6" t="s">
+      <c r="C23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
+      <c r="A24" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
+      <c r="A25" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="1"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="1"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="1"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
+      <c r="A26" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" s="7"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>